<commit_message>
Update results: revise CEA/OWSA outputs; add PSA outputs and CE plane visuals
</commit_message>
<xml_diff>
--- a/rsv_cea_results.xlsx
+++ b/rsv_cea_results.xlsx
@@ -1,98 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10215"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://fandtlabs-my.sharepoint.com/personal/jefferson_fandtlabs_com/Documents/Academic/Course Content/Economic Evaluation 3/rsv-vaccination-envaluation/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="11_EC68FDCE8F79A8D366075C52F3D99A770587C71A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CA445E8C-36FD-8B46-9164-00C01F907B2C}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="600" windowWidth="16100" windowHeight="9660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="22">
-  <si>
-    <t>Scenario</t>
-  </si>
-  <si>
-    <t>Total_Periods</t>
-  </si>
-  <si>
-    <t>Total Cost (Millions)</t>
-  </si>
-  <si>
-    <t>Total QALY (Millions)</t>
-  </si>
-  <si>
-    <t>Incremental Cost (Millions)</t>
-  </si>
-  <si>
-    <t>Incremental QALY (Millions)</t>
-  </si>
-  <si>
-    <t>ICER ($/QALY)</t>
-  </si>
-  <si>
-    <t>Standard of Care</t>
-  </si>
-  <si>
-    <t>$717,536.37</t>
-  </si>
-  <si>
-    <t>660.44</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>Abrysvo</t>
-  </si>
-  <si>
-    <t>$683,436.19</t>
-  </si>
-  <si>
-    <t>660.63</t>
-  </si>
-  <si>
-    <t>$-34,100.18</t>
-  </si>
-  <si>
-    <t>0.19</t>
-  </si>
-  <si>
-    <t>$-183,055.28</t>
-  </si>
-  <si>
-    <t>Arexvy</t>
-  </si>
-  <si>
-    <t>$680,396.58</t>
-  </si>
-  <si>
-    <t>$-3,039.61</t>
-  </si>
-  <si>
-    <t>0.00</t>
-  </si>
-  <si>
-    <t>$-1,318,307.95</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -140,21 +63,13 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -192,7 +107,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -226,7 +141,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -261,10 +175,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -437,105 +350,150 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="3" max="3" width="16.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="22.33203125" bestFit="1" customWidth="1"/>
-  </cols>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Total_Periods</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Total Cost (Millions)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Total QALY (Millions)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Incremental Cost (Millions)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Incremental QALY (Millions)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>ICER ($/QALY)</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>7</v>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Standard of Care</t>
+        </is>
       </c>
       <c r="B2">
         <v>12878</v>
       </c>
-      <c r="C2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G2" t="s">
-        <v>10</v>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>$717,536.37</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>660.44</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>11</v>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Abrysvo</t>
+        </is>
       </c>
       <c r="B3">
         <v>12500</v>
       </c>
-      <c r="C3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E3" t="s">
-        <v>14</v>
-      </c>
-      <c r="F3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G3" t="s">
-        <v>16</v>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>$683,436.19</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>660.63</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>$-34,100.18</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>0.19</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>$-183,055.28</t>
+        </is>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>17</v>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Arexvy</t>
+        </is>
       </c>
       <c r="B4">
         <v>12500</v>
       </c>
-      <c r="C4" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" t="s">
-        <v>13</v>
-      </c>
-      <c r="E4" t="s">
-        <v>19</v>
-      </c>
-      <c r="F4" t="s">
-        <v>20</v>
-      </c>
-      <c r="G4" t="s">
-        <v>21</v>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>$680,396.58</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>660.63</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>$-3,039.61</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>$-1,318,307.95</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update "healthcare" perspective logic to exclude all non-medical costs, revise outputs, and add societal perspective result files
</commit_message>
<xml_diff>
--- a/rsv_cea_results.xlsx
+++ b/rsv_cea_results.xlsx
@@ -402,7 +402,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>$717,536.37</t>
+          <t>$27.88</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -437,7 +437,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>$683,436.19</t>
+          <t>$21,496.58</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -447,7 +447,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>$-34,100.18</t>
+          <t>$21,468.69</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -457,7 +457,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>$-183,055.28</t>
+          <t>$115,247.41</t>
         </is>
       </c>
     </row>
@@ -472,7 +472,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>$680,396.58</t>
+          <t>$19,047.87</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -482,7 +482,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>$-3,039.61</t>
+          <t>$-2,448.71</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -492,7 +492,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>$-1,318,307.95</t>
+          <t>$-1,062,029.23</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add RSV vaccination cost-effectiveness analysis model with simulation framework, parameter definitions, and validation functions; initialize key transitions, outcomes, and cost perspectives.
</commit_message>
<xml_diff>
--- a/rsv_cea_results.xlsx
+++ b/rsv_cea_results.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -362,32 +362,42 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Total_Periods</t>
+          <t>Total Cost (Millions)</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Total Cost (Millions)</t>
+          <t>Total QALY (Millions)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Total QALY (Millions)</t>
+          <t>NHB @$100k (Millions)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Incremental Cost (Millions)</t>
+          <t>NMB @$100k (Millions)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Incremental QALY (Millions)</t>
+          <t>INMB @$100k (Millions)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>ICER ($/QALY)</t>
+          <t>NHB @$150k (Millions)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>NMB @$150k (Millions)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>INMB @$150k (Millions)</t>
         </is>
       </c>
     </row>
@@ -397,30 +407,42 @@
           <t>Standard of Care</t>
         </is>
       </c>
-      <c r="B2">
-        <v>12878</v>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>$717,536.33</t>
+        </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>$27.88</t>
+          <t>660.44</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>660.44</t>
+          <t>653.27</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>$65,326,619.18</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="G2" t="inlineStr">
+        <is>
+          <t>655.66</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>$98,348,696.94</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -429,70 +451,94 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Abrysvo</t>
-        </is>
-      </c>
-      <c r="B3">
-        <v>12500</v>
+          <t>Arexvy</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>$680,396.55</t>
+        </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>$21,496.58</t>
+          <t>660.63</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>660.63</t>
+          <t>653.83</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>$21,468.69</t>
+          <t>$65,382,617.79</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0.19</t>
+          <t>$55,998.61</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>$115,247.41</t>
+          <t>656.09</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>$98,414,124.96</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>$65,428.02</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Arexvy</t>
-        </is>
-      </c>
-      <c r="B4">
-        <v>12500</v>
+          <t>Abrysvo</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>$683,436.16</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>$19,047.87</t>
+          <t>660.63</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>660.63</t>
+          <t>653.79</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>$-2,448.71</t>
+          <t>$65,379,347.61</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>$52,728.43</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>$-1,062,029.23</t>
+          <t>656.07</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>$98,410,739.50</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>$62,042.56</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Convert cost metrics from millions to billions across all RSV model outputs, update tornado diagram logic for improved readability, and regenerate results and visuals, including Excel files and plots.
</commit_message>
<xml_diff>
--- a/rsv_cea_results.xlsx
+++ b/rsv_cea_results.xlsx
@@ -362,7 +362,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Total Cost (Millions)</t>
+          <t>Total Cost (Billions)</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -377,12 +377,12 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>NMB @$100k (Millions)</t>
+          <t>NMB @$100k (Billions)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>INMB @$100k (Millions)</t>
+          <t>INMB @$100k (Billions)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -392,12 +392,12 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>NMB @$150k (Millions)</t>
+          <t>NMB @$150k (Billions)</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>INMB @$150k (Millions)</t>
+          <t>INMB @$150k (Billions)</t>
         </is>
       </c>
     </row>
@@ -409,7 +409,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>$717,536.33</t>
+          <t>$717.54</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -424,7 +424,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>$65,326,619.18</t>
+          <t>$65,326.62</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -439,7 +439,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>$98,348,696.94</t>
+          <t>$98,348.70</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -456,7 +456,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>$680,396.55</t>
+          <t>$680.40</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -471,12 +471,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>$65,382,617.79</t>
+          <t>$65,382.62</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>$55,998.61</t>
+          <t>$56.00</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -486,12 +486,12 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>$98,414,124.96</t>
+          <t>$98,414.12</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>$65,428.02</t>
+          <t>$65.43</t>
         </is>
       </c>
     </row>
@@ -503,7 +503,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>$683,436.16</t>
+          <t>$683.44</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -518,12 +518,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>$65,379,347.61</t>
+          <t>$65,379.35</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>$52,728.43</t>
+          <t>$52.73</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -533,12 +533,12 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>$98,410,739.50</t>
+          <t>$98,410.74</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>$62,042.56</t>
+          <t>$62.04</t>
         </is>
       </c>
     </row>

</xml_diff>